<commit_message>
Atualiza planilha de disponibilidade - 03/06/2026 11:17
</commit_message>
<xml_diff>
--- a/disponibilidade.xlsx
+++ b/disponibilidade.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rafael.germano\Documents\Rafael Germano\Codex\2026-05-19\app disponiblidade\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EDF6F0A-CEB2-47A8-9B8E-D1168A02BD2D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2E9B730-9C71-473F-AB0F-0F348C02682A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -413,6 +413,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -423,9 +426,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -772,7 +772,7 @@
         <v>21</v>
       </c>
       <c r="B6" s="14">
-        <v>750</v>
+        <v>250</v>
       </c>
       <c r="F6" s="7" t="s">
         <v>21</v>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="B62" s="15">
         <f>SUM(B63:B64)</f>
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F62" s="9" t="s">
         <v>25</v>
@@ -1672,9 +1672,7 @@
       <c r="A63" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B63" s="15">
-        <v>30</v>
-      </c>
+      <c r="B63" s="15"/>
       <c r="F63" s="9" t="s">
         <v>21</v>
       </c>
@@ -2116,7 +2114,7 @@
       </c>
       <c r="B89" s="13">
         <f>SUM(B53,B56,B59,B62,B65,B68,B71,B74,B77,B80,B83,B86)</f>
-        <v>730</v>
+        <v>700</v>
       </c>
       <c r="F89" s="8" t="s">
         <v>34</v>
@@ -2180,19 +2178,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="21" t="s">
         <v>15</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
       <c r="D1" s="20"/>
-      <c r="F1" s="25" t="s">
+      <c r="F1" s="21" t="s">
         <v>15</v>
       </c>
       <c r="G1" s="20"/>
       <c r="H1" s="20"/>
       <c r="I1" s="20"/>
-      <c r="K1" s="25" t="s">
+      <c r="K1" s="21" t="s">
         <v>15</v>
       </c>
       <c r="L1" s="20"/>
@@ -2200,19 +2198,19 @@
       <c r="N1" s="20"/>
     </row>
     <row r="2" spans="1:14" ht="15" customHeight="1">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="21" t="s">
         <v>36</v>
       </c>
       <c r="B2" s="20"/>
       <c r="C2" s="20"/>
       <c r="D2" s="20"/>
-      <c r="F2" s="25" t="s">
+      <c r="F2" s="21" t="s">
         <v>36</v>
       </c>
       <c r="G2" s="20"/>
       <c r="H2" s="20"/>
       <c r="I2" s="20"/>
-      <c r="K2" s="25" t="s">
+      <c r="K2" s="21" t="s">
         <v>36</v>
       </c>
       <c r="L2" s="20"/>
@@ -2234,27 +2232,27 @@
       <c r="N3" s="9"/>
     </row>
     <row r="4" spans="1:14" ht="15" customHeight="1">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="24" t="s">
         <v>37</v>
       </c>
       <c r="B4" s="20"/>
-      <c r="C4" s="23" t="s">
+      <c r="C4" s="24" t="s">
         <v>38</v>
       </c>
       <c r="D4" s="20"/>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="24" t="s">
         <v>37</v>
       </c>
       <c r="G4" s="20"/>
-      <c r="H4" s="23" t="s">
+      <c r="H4" s="24" t="s">
         <v>39</v>
       </c>
       <c r="I4" s="20"/>
-      <c r="K4" s="23" t="s">
+      <c r="K4" s="24" t="s">
         <v>37</v>
       </c>
       <c r="L4" s="20"/>
-      <c r="M4" s="23" t="s">
+      <c r="M4" s="24" t="s">
         <v>40</v>
       </c>
       <c r="N4" s="20"/>
@@ -2263,7 +2261,7 @@
       <c r="A5" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="22">
+      <c r="B5" s="23">
         <v>559</v>
       </c>
       <c r="C5" s="20"/>
@@ -2271,13 +2269,13 @@
       <c r="F5" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G5" s="22"/>
+      <c r="G5" s="23"/>
       <c r="H5" s="20"/>
       <c r="I5" s="20"/>
       <c r="K5" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="L5" s="22"/>
+      <c r="L5" s="23"/>
       <c r="M5" s="20"/>
       <c r="N5" s="20"/>
     </row>
@@ -2285,7 +2283,7 @@
       <c r="A6" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="21">
+      <c r="B6" s="22">
         <v>2345</v>
       </c>
       <c r="C6" s="20"/>
@@ -2293,13 +2291,13 @@
       <c r="F6" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="G6" s="21"/>
+      <c r="G6" s="22"/>
       <c r="H6" s="20"/>
       <c r="I6" s="20"/>
       <c r="K6" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="L6" s="21"/>
+      <c r="L6" s="22"/>
       <c r="M6" s="20"/>
       <c r="N6" s="20"/>
     </row>
@@ -2307,7 +2305,7 @@
       <c r="A7" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="22">
+      <c r="B7" s="23">
         <v>1762</v>
       </c>
       <c r="C7" s="20"/>
@@ -2315,13 +2313,13 @@
       <c r="F7" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G7" s="22"/>
+      <c r="G7" s="23"/>
       <c r="H7" s="20"/>
       <c r="I7" s="20"/>
       <c r="K7" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="L7" s="22"/>
+      <c r="L7" s="23"/>
       <c r="M7" s="20"/>
       <c r="N7" s="20"/>
     </row>
@@ -2329,7 +2327,7 @@
       <c r="A8" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="21">
+      <c r="B8" s="22">
         <v>2425</v>
       </c>
       <c r="C8" s="20"/>
@@ -2337,13 +2335,13 @@
       <c r="F8" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="G8" s="21"/>
+      <c r="G8" s="22"/>
       <c r="H8" s="20"/>
       <c r="I8" s="20"/>
       <c r="K8" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="L8" s="21"/>
+      <c r="L8" s="22"/>
       <c r="M8" s="20"/>
       <c r="N8" s="20"/>
     </row>
@@ -2351,7 +2349,7 @@
       <c r="A9" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="22">
+      <c r="B9" s="23">
         <v>798</v>
       </c>
       <c r="C9" s="20"/>
@@ -2359,13 +2357,13 @@
       <c r="F9" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G9" s="22"/>
+      <c r="G9" s="23"/>
       <c r="H9" s="20"/>
       <c r="I9" s="20"/>
       <c r="K9" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="L9" s="22"/>
+      <c r="L9" s="23"/>
       <c r="M9" s="20"/>
       <c r="N9" s="20"/>
     </row>
@@ -2373,7 +2371,7 @@
       <c r="A10" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B10" s="21">
+      <c r="B10" s="22">
         <v>160</v>
       </c>
       <c r="C10" s="20"/>
@@ -2381,13 +2379,13 @@
       <c r="F10" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="G10" s="21"/>
+      <c r="G10" s="22"/>
       <c r="H10" s="20"/>
       <c r="I10" s="20"/>
       <c r="K10" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="L10" s="21"/>
+      <c r="L10" s="22"/>
       <c r="M10" s="20"/>
       <c r="N10" s="20"/>
     </row>
@@ -2395,7 +2393,7 @@
       <c r="A11" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="24">
+      <c r="B11" s="25">
         <f>SUM(B5:B10)</f>
         <v>8049</v>
       </c>
@@ -2404,7 +2402,7 @@
       <c r="F11" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="G11" s="24">
+      <c r="G11" s="25">
         <f>SUM(G5:G10)</f>
         <v>0</v>
       </c>
@@ -2413,7 +2411,7 @@
       <c r="K11" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="L11" s="24">
+      <c r="L11" s="25">
         <f>SUM(L5:L10)</f>
         <v>0</v>
       </c>
@@ -2449,19 +2447,19 @@
       <c r="N13" s="9"/>
     </row>
     <row r="25" spans="1:14" ht="15" customHeight="1">
-      <c r="A25" s="25" t="s">
+      <c r="A25" s="21" t="s">
         <v>15</v>
       </c>
       <c r="B25" s="20"/>
       <c r="C25" s="20"/>
       <c r="D25" s="20"/>
-      <c r="F25" s="25" t="s">
+      <c r="F25" s="21" t="s">
         <v>15</v>
       </c>
       <c r="G25" s="20"/>
       <c r="H25" s="20"/>
       <c r="I25" s="20"/>
-      <c r="K25" s="25" t="s">
+      <c r="K25" s="21" t="s">
         <v>15</v>
       </c>
       <c r="L25" s="20"/>
@@ -2469,19 +2467,19 @@
       <c r="N25" s="20"/>
     </row>
     <row r="26" spans="1:14" ht="15" customHeight="1">
-      <c r="A26" s="25" t="s">
+      <c r="A26" s="21" t="s">
         <v>36</v>
       </c>
       <c r="B26" s="20"/>
       <c r="C26" s="20"/>
       <c r="D26" s="20"/>
-      <c r="F26" s="25" t="s">
+      <c r="F26" s="21" t="s">
         <v>36</v>
       </c>
       <c r="G26" s="20"/>
       <c r="H26" s="20"/>
       <c r="I26" s="20"/>
-      <c r="K26" s="25" t="s">
+      <c r="K26" s="21" t="s">
         <v>36</v>
       </c>
       <c r="L26" s="20"/>
@@ -2503,27 +2501,27 @@
       <c r="N27" s="9"/>
     </row>
     <row r="28" spans="1:14" ht="15" customHeight="1">
-      <c r="A28" s="23" t="s">
+      <c r="A28" s="24" t="s">
         <v>47</v>
       </c>
       <c r="B28" s="20"/>
-      <c r="C28" s="23" t="s">
+      <c r="C28" s="24" t="s">
         <v>38</v>
       </c>
       <c r="D28" s="20"/>
-      <c r="F28" s="23" t="s">
+      <c r="F28" s="24" t="s">
         <v>47</v>
       </c>
       <c r="G28" s="20"/>
-      <c r="H28" s="23" t="s">
+      <c r="H28" s="24" t="s">
         <v>39</v>
       </c>
       <c r="I28" s="20"/>
-      <c r="K28" s="23" t="s">
+      <c r="K28" s="24" t="s">
         <v>47</v>
       </c>
       <c r="L28" s="20"/>
-      <c r="M28" s="23" t="s">
+      <c r="M28" s="24" t="s">
         <v>40</v>
       </c>
       <c r="N28" s="20"/>
@@ -2532,7 +2530,7 @@
       <c r="A29" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B29" s="22">
+      <c r="B29" s="23">
         <v>0</v>
       </c>
       <c r="C29" s="20"/>
@@ -2540,13 +2538,13 @@
       <c r="F29" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G29" s="22"/>
+      <c r="G29" s="23"/>
       <c r="H29" s="20"/>
       <c r="I29" s="20"/>
       <c r="K29" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="L29" s="22">
+      <c r="L29" s="23">
         <v>9</v>
       </c>
       <c r="M29" s="20"/>
@@ -2556,7 +2554,7 @@
       <c r="A30" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B30" s="21">
+      <c r="B30" s="22">
         <v>0</v>
       </c>
       <c r="C30" s="20"/>
@@ -2564,13 +2562,13 @@
       <c r="F30" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="G30" s="21"/>
+      <c r="G30" s="22"/>
       <c r="H30" s="20"/>
       <c r="I30" s="20"/>
       <c r="K30" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="L30" s="21">
+      <c r="L30" s="22">
         <v>359</v>
       </c>
       <c r="M30" s="20"/>
@@ -2580,7 +2578,7 @@
       <c r="A31" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B31" s="22">
+      <c r="B31" s="23">
         <v>0</v>
       </c>
       <c r="C31" s="20"/>
@@ -2588,13 +2586,13 @@
       <c r="F31" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G31" s="22"/>
+      <c r="G31" s="23"/>
       <c r="H31" s="20"/>
       <c r="I31" s="20"/>
       <c r="K31" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="L31" s="22">
+      <c r="L31" s="23">
         <v>1024</v>
       </c>
       <c r="M31" s="20"/>
@@ -2604,7 +2602,7 @@
       <c r="A32" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B32" s="21">
+      <c r="B32" s="22">
         <v>350</v>
       </c>
       <c r="C32" s="20"/>
@@ -2612,13 +2610,13 @@
       <c r="F32" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="G32" s="21"/>
+      <c r="G32" s="22"/>
       <c r="H32" s="20"/>
       <c r="I32" s="20"/>
       <c r="K32" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="L32" s="21">
+      <c r="L32" s="22">
         <v>1036</v>
       </c>
       <c r="M32" s="20"/>
@@ -2628,7 +2626,7 @@
       <c r="A33" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B33" s="22">
+      <c r="B33" s="23">
         <v>603</v>
       </c>
       <c r="C33" s="20"/>
@@ -2636,13 +2634,13 @@
       <c r="F33" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G33" s="22"/>
+      <c r="G33" s="23"/>
       <c r="H33" s="20"/>
       <c r="I33" s="20"/>
       <c r="K33" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="L33" s="22">
+      <c r="L33" s="23">
         <v>197</v>
       </c>
       <c r="M33" s="20"/>
@@ -2652,7 +2650,7 @@
       <c r="A34" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B34" s="21">
+      <c r="B34" s="22">
         <v>50</v>
       </c>
       <c r="C34" s="20"/>
@@ -2660,13 +2658,13 @@
       <c r="F34" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="G34" s="21"/>
+      <c r="G34" s="22"/>
       <c r="H34" s="20"/>
       <c r="I34" s="20"/>
       <c r="K34" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="L34" s="21"/>
+      <c r="L34" s="22"/>
       <c r="M34" s="20"/>
       <c r="N34" s="20"/>
     </row>
@@ -2674,7 +2672,7 @@
       <c r="A35" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B35" s="24">
+      <c r="B35" s="25">
         <f>SUM(B29:B34)</f>
         <v>1003</v>
       </c>
@@ -2683,7 +2681,7 @@
       <c r="F35" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="G35" s="24">
+      <c r="G35" s="25">
         <f>SUM(G29:G34)</f>
         <v>0</v>
       </c>
@@ -2692,7 +2690,7 @@
       <c r="K35" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="L35" s="24">
+      <c r="L35" s="25">
         <f>SUM(L29:L34)</f>
         <v>2625</v>
       </c>
@@ -2729,13 +2727,49 @@
     </row>
   </sheetData>
   <mergeCells count="66">
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="L32:N32"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="L29:N29"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="L5:N5"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="G35:I35"/>
+    <mergeCell ref="L31:N31"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="L34:N34"/>
+    <mergeCell ref="G29:I29"/>
+    <mergeCell ref="L33:N33"/>
+    <mergeCell ref="L35:N35"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="G30:I30"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="L30:N30"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="G34:I34"/>
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="L10:N10"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="K25:N25"/>
+    <mergeCell ref="L9:N9"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="L6:N6"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="L8:N8"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="G11:I11"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="L11:N11"/>
@@ -2752,49 +2786,13 @@
     <mergeCell ref="K2:N2"/>
     <mergeCell ref="K4:L4"/>
     <mergeCell ref="G7:I7"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="L10:N10"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="K25:N25"/>
-    <mergeCell ref="L9:N9"/>
-    <mergeCell ref="F25:I25"/>
-    <mergeCell ref="L6:N6"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="L8:N8"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="G35:I35"/>
-    <mergeCell ref="L31:N31"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="L34:N34"/>
-    <mergeCell ref="G29:I29"/>
-    <mergeCell ref="L33:N33"/>
-    <mergeCell ref="L35:N35"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="G30:I30"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="G33:I33"/>
-    <mergeCell ref="L30:N30"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="G34:I34"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B33:D33"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="L29:N29"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="L5:N5"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="L32:N32"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="C28:D28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2810,7 +2808,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="21" t="s">
         <v>15</v>
       </c>
       <c r="B1" s="20"/>
@@ -2818,7 +2816,7 @@
       <c r="D1" s="20"/>
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="21" t="s">
         <v>36</v>
       </c>
       <c r="B2" s="20"/>
@@ -2832,11 +2830,11 @@
       <c r="D3" s="9"/>
     </row>
     <row r="4" spans="1:4" ht="15" customHeight="1">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="24" t="s">
         <v>19</v>
       </c>
       <c r="B4" s="20"/>
-      <c r="C4" s="23" t="s">
+      <c r="C4" s="24" t="s">
         <v>48</v>
       </c>
       <c r="D4" s="20"/>
@@ -2845,7 +2843,7 @@
       <c r="A5" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B5" s="22"/>
+      <c r="B5" s="23"/>
       <c r="C5" s="20"/>
       <c r="D5" s="20"/>
     </row>
@@ -2853,7 +2851,7 @@
       <c r="A6" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B6" s="21"/>
+      <c r="B6" s="22"/>
       <c r="C6" s="20"/>
       <c r="D6" s="20"/>
     </row>
@@ -2861,7 +2859,7 @@
       <c r="A7" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="22"/>
+      <c r="B7" s="23"/>
       <c r="C7" s="20"/>
       <c r="D7" s="20"/>
     </row>
@@ -2869,7 +2867,7 @@
       <c r="A8" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B8" s="21"/>
+      <c r="B8" s="22"/>
       <c r="C8" s="20"/>
       <c r="D8" s="20"/>
     </row>
@@ -2877,7 +2875,7 @@
       <c r="A9" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="24">
+      <c r="B9" s="25">
         <f>SUM(B5:B8)</f>
         <v>0</v>
       </c>
@@ -2926,19 +2924,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="21" t="s">
         <v>15</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
       <c r="D1" s="20"/>
-      <c r="F1" s="25" t="s">
+      <c r="F1" s="21" t="s">
         <v>15</v>
       </c>
       <c r="G1" s="20"/>
       <c r="H1" s="20"/>
       <c r="I1" s="20"/>
-      <c r="K1" s="25" t="s">
+      <c r="K1" s="21" t="s">
         <v>15</v>
       </c>
       <c r="L1" s="20"/>
@@ -2946,19 +2944,19 @@
       <c r="N1" s="20"/>
     </row>
     <row r="2" spans="1:14" ht="15" customHeight="1">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="21" t="s">
         <v>36</v>
       </c>
       <c r="B2" s="20"/>
       <c r="C2" s="20"/>
       <c r="D2" s="20"/>
-      <c r="F2" s="25" t="s">
+      <c r="F2" s="21" t="s">
         <v>36</v>
       </c>
       <c r="G2" s="20"/>
       <c r="H2" s="20"/>
       <c r="I2" s="20"/>
-      <c r="K2" s="25" t="s">
+      <c r="K2" s="21" t="s">
         <v>36</v>
       </c>
       <c r="L2" s="20"/>
@@ -2980,27 +2978,27 @@
       <c r="N3" s="9"/>
     </row>
     <row r="4" spans="1:14" ht="15" customHeight="1">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="24" t="s">
         <v>37</v>
       </c>
       <c r="B4" s="20"/>
-      <c r="C4" s="23" t="s">
+      <c r="C4" s="24" t="s">
         <v>53</v>
       </c>
       <c r="D4" s="20"/>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="24" t="s">
         <v>37</v>
       </c>
       <c r="G4" s="20"/>
-      <c r="H4" s="23" t="s">
+      <c r="H4" s="24" t="s">
         <v>54</v>
       </c>
       <c r="I4" s="20"/>
-      <c r="K4" s="23" t="s">
+      <c r="K4" s="24" t="s">
         <v>37</v>
       </c>
       <c r="L4" s="20"/>
-      <c r="M4" s="23" t="s">
+      <c r="M4" s="24" t="s">
         <v>55</v>
       </c>
       <c r="N4" s="20"/>
@@ -3009,19 +3007,19 @@
       <c r="A5" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="22"/>
+      <c r="B5" s="23"/>
       <c r="C5" s="20"/>
       <c r="D5" s="20"/>
       <c r="F5" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="G5" s="22"/>
+      <c r="G5" s="23"/>
       <c r="H5" s="20"/>
       <c r="I5" s="20"/>
       <c r="K5" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="L5" s="22"/>
+      <c r="L5" s="23"/>
       <c r="M5" s="20"/>
       <c r="N5" s="20"/>
     </row>
@@ -3029,19 +3027,19 @@
       <c r="A6" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="21"/>
+      <c r="B6" s="22"/>
       <c r="C6" s="20"/>
       <c r="D6" s="20"/>
       <c r="F6" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="G6" s="21"/>
+      <c r="G6" s="22"/>
       <c r="H6" s="20"/>
       <c r="I6" s="20"/>
       <c r="K6" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="L6" s="21"/>
+      <c r="L6" s="22"/>
       <c r="M6" s="20"/>
       <c r="N6" s="20"/>
     </row>
@@ -3049,19 +3047,19 @@
       <c r="A7" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B7" s="22"/>
+      <c r="B7" s="23"/>
       <c r="C7" s="20"/>
       <c r="D7" s="20"/>
       <c r="F7" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="G7" s="22"/>
+      <c r="G7" s="23"/>
       <c r="H7" s="20"/>
       <c r="I7" s="20"/>
       <c r="K7" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="L7" s="22"/>
+      <c r="L7" s="23"/>
       <c r="M7" s="20"/>
       <c r="N7" s="20"/>
     </row>
@@ -3069,19 +3067,19 @@
       <c r="A8" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B8" s="21"/>
+      <c r="B8" s="22"/>
       <c r="C8" s="20"/>
       <c r="D8" s="20"/>
       <c r="F8" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G8" s="21"/>
+      <c r="G8" s="22"/>
       <c r="H8" s="20"/>
       <c r="I8" s="20"/>
       <c r="K8" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="L8" s="21"/>
+      <c r="L8" s="22"/>
       <c r="M8" s="20"/>
       <c r="N8" s="20"/>
     </row>
@@ -3089,19 +3087,19 @@
       <c r="A9" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B9" s="22"/>
+      <c r="B9" s="23"/>
       <c r="C9" s="20"/>
       <c r="D9" s="20"/>
       <c r="F9" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="G9" s="22"/>
+      <c r="G9" s="23"/>
       <c r="H9" s="20"/>
       <c r="I9" s="20"/>
       <c r="K9" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="L9" s="22"/>
+      <c r="L9" s="23"/>
       <c r="M9" s="20"/>
       <c r="N9" s="20"/>
     </row>
@@ -3109,7 +3107,7 @@
       <c r="A10" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B10" s="21">
+      <c r="B10" s="22">
         <v>0</v>
       </c>
       <c r="C10" s="20"/>
@@ -3117,13 +3115,13 @@
       <c r="F10" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="G10" s="21"/>
+      <c r="G10" s="22"/>
       <c r="H10" s="20"/>
       <c r="I10" s="20"/>
       <c r="K10" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L10" s="21"/>
+      <c r="L10" s="22"/>
       <c r="M10" s="20"/>
       <c r="N10" s="20"/>
     </row>
@@ -3131,7 +3129,7 @@
       <c r="A11" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="22">
+      <c r="B11" s="23">
         <v>700</v>
       </c>
       <c r="C11" s="20"/>
@@ -3139,13 +3137,13 @@
       <c r="F11" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="G11" s="22"/>
+      <c r="G11" s="23"/>
       <c r="H11" s="20"/>
       <c r="I11" s="20"/>
       <c r="K11" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="L11" s="22"/>
+      <c r="L11" s="23"/>
       <c r="M11" s="20"/>
       <c r="N11" s="20"/>
     </row>
@@ -3153,7 +3151,7 @@
       <c r="A12" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B12" s="21">
+      <c r="B12" s="22">
         <v>500</v>
       </c>
       <c r="C12" s="20"/>
@@ -3161,13 +3159,13 @@
       <c r="F12" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="G12" s="21"/>
+      <c r="G12" s="22"/>
       <c r="H12" s="20"/>
       <c r="I12" s="20"/>
       <c r="K12" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="L12" s="21"/>
+      <c r="L12" s="22"/>
       <c r="M12" s="20"/>
       <c r="N12" s="20"/>
     </row>
@@ -3175,7 +3173,7 @@
       <c r="A13" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="24">
+      <c r="B13" s="25">
         <f>SUM(B5:B12)</f>
         <v>1200</v>
       </c>
@@ -3184,7 +3182,7 @@
       <c r="F13" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="G13" s="24">
+      <c r="G13" s="25">
         <f>SUM(G5:G12)</f>
         <v>0</v>
       </c>
@@ -3193,7 +3191,7 @@
       <c r="K13" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="L13" s="24">
+      <c r="L13" s="25">
         <f>SUM(L5:L12)</f>
         <v>0</v>
       </c>
@@ -3229,19 +3227,19 @@
       <c r="N15" s="9"/>
     </row>
     <row r="25" spans="1:14" ht="15" customHeight="1">
-      <c r="A25" s="25" t="s">
+      <c r="A25" s="21" t="s">
         <v>15</v>
       </c>
       <c r="B25" s="20"/>
       <c r="C25" s="20"/>
       <c r="D25" s="20"/>
-      <c r="F25" s="25" t="s">
+      <c r="F25" s="21" t="s">
         <v>15</v>
       </c>
       <c r="G25" s="20"/>
       <c r="H25" s="20"/>
       <c r="I25" s="20"/>
-      <c r="K25" s="25" t="s">
+      <c r="K25" s="21" t="s">
         <v>15</v>
       </c>
       <c r="L25" s="20"/>
@@ -3249,19 +3247,19 @@
       <c r="N25" s="20"/>
     </row>
     <row r="26" spans="1:14" ht="15" customHeight="1">
-      <c r="A26" s="25" t="s">
+      <c r="A26" s="21" t="s">
         <v>36</v>
       </c>
       <c r="B26" s="20"/>
       <c r="C26" s="20"/>
       <c r="D26" s="20"/>
-      <c r="F26" s="25" t="s">
+      <c r="F26" s="21" t="s">
         <v>36</v>
       </c>
       <c r="G26" s="20"/>
       <c r="H26" s="20"/>
       <c r="I26" s="20"/>
-      <c r="K26" s="25" t="s">
+      <c r="K26" s="21" t="s">
         <v>36</v>
       </c>
       <c r="L26" s="20"/>
@@ -3283,27 +3281,27 @@
       <c r="N27" s="9"/>
     </row>
     <row r="28" spans="1:14" ht="15" customHeight="1">
-      <c r="A28" s="23" t="s">
+      <c r="A28" s="24" t="s">
         <v>47</v>
       </c>
       <c r="B28" s="20"/>
-      <c r="C28" s="23" t="s">
+      <c r="C28" s="24" t="s">
         <v>53</v>
       </c>
       <c r="D28" s="20"/>
-      <c r="F28" s="23" t="s">
+      <c r="F28" s="24" t="s">
         <v>47</v>
       </c>
       <c r="G28" s="20"/>
-      <c r="H28" s="23" t="s">
+      <c r="H28" s="24" t="s">
         <v>54</v>
       </c>
       <c r="I28" s="20"/>
-      <c r="K28" s="23" t="s">
+      <c r="K28" s="24" t="s">
         <v>47</v>
       </c>
       <c r="L28" s="20"/>
-      <c r="M28" s="23" t="s">
+      <c r="M28" s="24" t="s">
         <v>55</v>
       </c>
       <c r="N28" s="20"/>
@@ -3312,19 +3310,19 @@
       <c r="A29" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B29" s="22"/>
+      <c r="B29" s="23"/>
       <c r="C29" s="20"/>
       <c r="D29" s="20"/>
       <c r="F29" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="G29" s="22"/>
+      <c r="G29" s="23"/>
       <c r="H29" s="20"/>
       <c r="I29" s="20"/>
       <c r="K29" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="L29" s="22"/>
+      <c r="L29" s="23"/>
       <c r="M29" s="20"/>
       <c r="N29" s="20"/>
     </row>
@@ -3332,19 +3330,19 @@
       <c r="A30" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B30" s="21"/>
+      <c r="B30" s="22"/>
       <c r="C30" s="20"/>
       <c r="D30" s="20"/>
       <c r="F30" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="G30" s="21"/>
+      <c r="G30" s="22"/>
       <c r="H30" s="20"/>
       <c r="I30" s="20"/>
       <c r="K30" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="L30" s="21"/>
+      <c r="L30" s="22"/>
       <c r="M30" s="20"/>
       <c r="N30" s="20"/>
     </row>
@@ -3352,19 +3350,19 @@
       <c r="A31" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B31" s="22"/>
+      <c r="B31" s="23"/>
       <c r="C31" s="20"/>
       <c r="D31" s="20"/>
       <c r="F31" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="G31" s="22"/>
+      <c r="G31" s="23"/>
       <c r="H31" s="20"/>
       <c r="I31" s="20"/>
       <c r="K31" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="L31" s="22"/>
+      <c r="L31" s="23"/>
       <c r="M31" s="20"/>
       <c r="N31" s="20"/>
     </row>
@@ -3372,19 +3370,19 @@
       <c r="A32" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B32" s="21"/>
+      <c r="B32" s="22"/>
       <c r="C32" s="20"/>
       <c r="D32" s="20"/>
       <c r="F32" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G32" s="21"/>
+      <c r="G32" s="22"/>
       <c r="H32" s="20"/>
       <c r="I32" s="20"/>
       <c r="K32" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="L32" s="21"/>
+      <c r="L32" s="22"/>
       <c r="M32" s="20"/>
       <c r="N32" s="20"/>
     </row>
@@ -3392,19 +3390,19 @@
       <c r="A33" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B33" s="22"/>
+      <c r="B33" s="23"/>
       <c r="C33" s="20"/>
       <c r="D33" s="20"/>
       <c r="F33" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="G33" s="22"/>
+      <c r="G33" s="23"/>
       <c r="H33" s="20"/>
       <c r="I33" s="20"/>
       <c r="K33" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="L33" s="22"/>
+      <c r="L33" s="23"/>
       <c r="M33" s="20"/>
       <c r="N33" s="20"/>
     </row>
@@ -3412,19 +3410,19 @@
       <c r="A34" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B34" s="21"/>
+      <c r="B34" s="22"/>
       <c r="C34" s="20"/>
       <c r="D34" s="20"/>
       <c r="F34" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="G34" s="21"/>
+      <c r="G34" s="22"/>
       <c r="H34" s="20"/>
       <c r="I34" s="20"/>
       <c r="K34" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L34" s="21"/>
+      <c r="L34" s="22"/>
       <c r="M34" s="20"/>
       <c r="N34" s="20"/>
     </row>
@@ -3432,19 +3430,19 @@
       <c r="A35" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B35" s="22"/>
+      <c r="B35" s="23"/>
       <c r="C35" s="20"/>
       <c r="D35" s="20"/>
       <c r="F35" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="G35" s="22"/>
+      <c r="G35" s="23"/>
       <c r="H35" s="20"/>
       <c r="I35" s="20"/>
       <c r="K35" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="L35" s="22"/>
+      <c r="L35" s="23"/>
       <c r="M35" s="20"/>
       <c r="N35" s="20"/>
     </row>
@@ -3452,19 +3450,19 @@
       <c r="A36" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B36" s="21"/>
+      <c r="B36" s="22"/>
       <c r="C36" s="20"/>
       <c r="D36" s="20"/>
       <c r="F36" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="G36" s="21"/>
+      <c r="G36" s="22"/>
       <c r="H36" s="20"/>
       <c r="I36" s="20"/>
       <c r="K36" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="L36" s="21"/>
+      <c r="L36" s="22"/>
       <c r="M36" s="20"/>
       <c r="N36" s="20"/>
     </row>
@@ -3472,7 +3470,7 @@
       <c r="A37" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B37" s="24">
+      <c r="B37" s="25">
         <f>SUM(B29:B36)</f>
         <v>0</v>
       </c>
@@ -3481,7 +3479,7 @@
       <c r="F37" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="G37" s="24">
+      <c r="G37" s="25">
         <f>SUM(G29:G36)</f>
         <v>0</v>
       </c>
@@ -3490,7 +3488,7 @@
       <c r="K37" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="L37" s="24">
+      <c r="L37" s="25">
         <f>SUM(L29:L36)</f>
         <v>0</v>
       </c>
@@ -3527,6 +3525,68 @@
     </row>
   </sheetData>
   <mergeCells count="78">
+    <mergeCell ref="G36:I36"/>
+    <mergeCell ref="L32:N32"/>
+    <mergeCell ref="L13:N13"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="G32:I32"/>
+    <mergeCell ref="L36:N36"/>
+    <mergeCell ref="L33:N33"/>
+    <mergeCell ref="L35:N35"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="L11:N11"/>
+    <mergeCell ref="K26:N26"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="L30:N30"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="L29:N29"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="L37:N37"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="L12:N12"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="G34:I34"/>
+    <mergeCell ref="K25:N25"/>
+    <mergeCell ref="G29:I29"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="G37:I37"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="L8:N8"/>
+    <mergeCell ref="G30:I30"/>
+    <mergeCell ref="G35:I35"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="L31:N31"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="F2:I2"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="K2:N2"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="L5:N5"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="F4:G4"/>
     <mergeCell ref="L34:N34"/>
     <mergeCell ref="L6:N6"/>
     <mergeCell ref="B33:D33"/>
@@ -3543,68 +3603,6 @@
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="A26:D26"/>
     <mergeCell ref="L9:N9"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="L31:N31"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="K2:N2"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="L5:N5"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="K1:N1"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="L37:N37"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="L12:N12"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="G34:I34"/>
-    <mergeCell ref="K25:N25"/>
-    <mergeCell ref="G29:I29"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="G31:I31"/>
-    <mergeCell ref="G37:I37"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="L8:N8"/>
-    <mergeCell ref="G30:I30"/>
-    <mergeCell ref="G35:I35"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="L30:N30"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="G33:I33"/>
-    <mergeCell ref="L29:N29"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="L11:N11"/>
-    <mergeCell ref="K26:N26"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="G36:I36"/>
-    <mergeCell ref="L32:N32"/>
-    <mergeCell ref="L13:N13"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="H28:I28"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="F25:I25"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="G32:I32"/>
-    <mergeCell ref="L36:N36"/>
-    <mergeCell ref="L33:N33"/>
-    <mergeCell ref="L35:N35"/>
-    <mergeCell ref="B34:D34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>